<commit_message>
Drop forced font in schedule workbook so emoji render
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MFonYWebf5mUtuPs646JGF
</commit_message>
<xml_diff>
--- a/投稿予約表.xlsx
+++ b/投稿予約表.xlsx
@@ -32,36 +32,29 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Yu Gothic"/>
       <b val="1"/>
       <sz val="14"/>
     </font>
     <font>
-      <name val="Yu Gothic"/>
       <color rgb="00555555"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Yu Gothic"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
     <font>
-      <name val="Yu Gothic"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Yu Gothic"/>
       <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Yu Gothic"/>
       <b val="1"/>
       <sz val="12"/>
     </font>
     <font>
-      <name val="Yu Gothic"/>
       <sz val="12"/>
     </font>
   </fonts>

</xml_diff>